<commit_message>
Resolver merge y guardar cambios
</commit_message>
<xml_diff>
--- a/InbentorioaE1T2.xlsx
+++ b/InbentorioaE1T2.xlsx
@@ -30255,12 +30255,9 @@
     </row>
     <row r="4" ht="25" customHeight="1" s="61"/>
     <row r="5" ht="26" customHeight="1" s="61">
-      <c r="B5" s="76" t="inlineStr">
-        <is>
-          <t>GORRIA
-(Muy Importante)
-Cuanto antes
-mejor</t>
+      <c r="B5" t="inlineStr" s="76">
+        <is>
+          <t>GORRIA</t>
         </is>
       </c>
       <c r="C5" s="77" t="inlineStr">
@@ -30403,12 +30400,9 @@
     </row>
     <row r="9" ht="22" customHeight="1" s="61"/>
     <row r="10" ht="26" customHeight="1" s="61">
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>LARANJA
-(Importante)
-Si es posible
-comprarlo bien</t>
+      <c r="B10" t="inlineStr" s="84">
+        <is>
+          <t>LARANJA</t>
         </is>
       </c>
       <c r="C10" s="77" t="inlineStr">
@@ -30550,12 +30544,9 @@
       </c>
     </row>
     <row r="15" ht="26" customHeight="1" s="61">
-      <c r="B15" s="88" t="inlineStr">
-        <is>
-          <t>BERDEA
-(Necesario)
-Sin máxima
-prioridad</t>
+      <c r="B15" t="inlineStr" s="88">
+        <is>
+          <t>BERDEA</t>
         </is>
       </c>
       <c r="C15" s="77" t="inlineStr">

</xml_diff>